<commit_message>
Add frontier model token-price time series tab
Add a chronological time series of published API token prices (USD/1M tokens)
for frontier/flagship model versions across OpenAI, Anthropic, Google, xAI and
DeepSeek, from GPT-4 (2023) to Claude Fable 5 (2026). Each launch and price
change is a separate row with input, output, 3:1 blended price, context window
and notes. Adds a new workbook tab, CSV export, provider pricing sources and
README docs.

Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/llm-token-pricing/LLM_Token_Pricing_Indices.xlsx
+++ b/llm-token-pricing/LLM_Token_Pricing_Indices.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="Indicators" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Silicon Data Suite" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Methodology" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Sources" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Frontier Price Time Series" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Silicon Data Suite" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Methodology" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Sources" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1685,6 +1686,2130 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J50"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>LLM Token Pricing Indices &amp; Indicators</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Aggregated reference - as of 2026-06-23. Point-in-time figures from public publisher materials.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Date (YYYY-MM)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Model version</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Input $/1M</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Output $/1M</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Blended 3:1 $/1M</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Context window</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>2023-03</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>GPT-4 (32K)</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>32K</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>Extended-context tier</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>2023-03</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>GPT-4 (8K)</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>8K</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>First GPT-4 API tier</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>2023-07</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Claude 2</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>100K</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>2023-11</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Claude 2.1</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>200K</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>2023-11</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>GPT-4 Turbo</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>128K</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>~3x cheaper than GPT-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>2023-12</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Gemini 1.0 Pro</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>32K</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>2024-02</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Gemini 1.5 Pro</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>1M</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>&lt;=128K tier; &gt;128K was $7/$21</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Claude 3 Opus</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>75</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>200K</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Claude 3 Sonnet</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Mid/frontier</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>200K</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>2024-05</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>GPT-4o</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>128K</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>2024-06</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Claude 3.5 Sonnet</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>200K</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>2024-08</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>GPT-4o</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>Price cut</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>4.375</v>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>128K</t>
+        </is>
+      </c>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>gpt-4o-2024-08-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>2024-09</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>o1-preview</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Reasoning</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>26.25</v>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>128K</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>2024-10</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Gemini 1.5 Pro</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Price cut</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H18" s="6" t="n">
+        <v>2.188</v>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>2M</t>
+        </is>
+      </c>
+      <c r="J18" s="6" t="inlineStr">
+        <is>
+          <t>&lt;=128K tier; ~64% cut</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2024-10</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>xAI</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Grok-2</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H19" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>128K</t>
+        </is>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>API GA</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>DeepSeek V3</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Open frontier</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H20" s="6" t="n">
+        <v>0.478</v>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>64K</t>
+        </is>
+      </c>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>Post-promo standard rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Gemini 2.0 Flash</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Frontier-adjacent</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>1M</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>o1</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Reasoning</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="H22" s="6" t="n">
+        <v>26.25</v>
+      </c>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>200K</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>DeepSeek R1</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Open reasoning</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>64K</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Claude 3.7 Sonnet</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>200K</t>
+        </is>
+      </c>
+      <c r="J24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>GPT-4.5</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Flagship (premium)</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>128K</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>Later deprecated</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>xAI</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Grok-3</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="H26" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>131K</t>
+        </is>
+      </c>
+      <c r="J26" s="6" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Gemini 2.5 Pro</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H27" s="4" t="n">
+        <v>3.438</v>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>1M</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>&lt;=200K tier; &gt;200K $2.50/$15</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>GPT-4.1</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="H28" s="6" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>1M</t>
+        </is>
+      </c>
+      <c r="J28" s="6" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>o3</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Reasoning</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G29" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="H29" s="4" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>200K</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Claude Opus 4</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="G30" s="6" t="n">
+        <v>75</v>
+      </c>
+      <c r="H30" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="I30" s="6" t="inlineStr">
+        <is>
+          <t>200K</t>
+        </is>
+      </c>
+      <c r="J30" s="6" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Claude Sonnet 4</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Mid/frontier</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G31" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="H31" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>200K</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>1M context added later</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>o3</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>Reasoning</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>Price cut</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G32" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="H32" s="6" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>200K</t>
+        </is>
+      </c>
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>~80% cut</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>o3-pro</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Reasoning (premium)</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="G33" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>200K</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>xAI</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>Grok-4</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G34" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="H34" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="I34" s="6" t="inlineStr">
+        <is>
+          <t>256K</t>
+        </is>
+      </c>
+      <c r="J34" s="6" t="inlineStr">
+        <is>
+          <t>Context later 2M</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>GPT-5</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G35" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H35" s="4" t="n">
+        <v>3.438</v>
+      </c>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>400K</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>Claude Sonnet 4.5</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>Mid/frontier</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G36" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="H36" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="I36" s="6" t="inlineStr">
+        <is>
+          <t>1M</t>
+        </is>
+      </c>
+      <c r="J36" s="6" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Claude Opus 4.6</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G37" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="H37" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>1M</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>Approx date; big drop vs Opus 4 ($15/$75)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Gemini 3 Flash</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>Frontier-adjacent</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G38" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="H38" s="6" t="n">
+        <v>1.125</v>
+      </c>
+      <c r="I38" s="6" t="inlineStr">
+        <is>
+          <t>1M</t>
+        </is>
+      </c>
+      <c r="J38" s="6" t="inlineStr">
+        <is>
+          <t>Approx date</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Gemini 3.1 Pro</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G39" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H39" s="4" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>2M</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>Preview; &lt;=200K tier, &gt;200K $4/$18</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>Claude Sonnet 4.6</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>Mid/frontier</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G40" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="H40" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="I40" s="6" t="inlineStr">
+        <is>
+          <t>1M</t>
+        </is>
+      </c>
+      <c r="J40" s="6" t="inlineStr">
+        <is>
+          <t>Approx date</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 Pro</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Open frontier</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="n">
+        <v>0.435</v>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="H41" s="4" t="n">
+        <v>0.544</v>
+      </c>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>1M</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>75% promo rate; original $1.74/$3.48</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>GPT-5.4</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G42" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="H42" s="6" t="n">
+        <v>5.625</v>
+      </c>
+      <c r="I42" s="6" t="inlineStr">
+        <is>
+          <t>1M</t>
+        </is>
+      </c>
+      <c r="J42" s="6" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>GPT-5.5</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G43" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="H43" s="4" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>1M</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>&gt;272K input billed at long-context premium</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>GPT-5.5 Pro</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>Flagship (premium)</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="G44" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="H44" s="6" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="I44" s="6" t="inlineStr">
+        <is>
+          <t>1M</t>
+        </is>
+      </c>
+      <c r="J44" s="6" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>xAI</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Grok 4.20</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G45" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="H45" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>2M</t>
+        </is>
+      </c>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>Reasoning &amp; non-reasoning same price</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>xAI</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>Grok 4.3</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G46" s="6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H46" s="6" t="n">
+        <v>1.562</v>
+      </c>
+      <c r="I46" s="6" t="inlineStr">
+        <is>
+          <t>1M</t>
+        </is>
+      </c>
+      <c r="J46" s="6" t="inlineStr">
+        <is>
+          <t>Released Apr 30 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Claude Opus 4.7</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G47" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="H47" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>1M</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>New tokenizer (~+35% tokens vs older)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>Claude Opus 4.8</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>Flagship</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G48" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="H48" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="I48" s="6" t="inlineStr">
+        <is>
+          <t>1M</t>
+        </is>
+      </c>
+      <c r="J48" s="6" t="inlineStr">
+        <is>
+          <t>Released May 28 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>Gemini 3.5 Flash</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>Frontier-adjacent</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G49" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="H49" s="4" t="n">
+        <v>3.375</v>
+      </c>
+      <c r="I49" s="4" t="inlineStr">
+        <is>
+          <t>1M</t>
+        </is>
+      </c>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>Released May 19 2026; beats 3.1 Pro on coding</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>Claude Fable 5</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>Flagship (frontier)</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="G50" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="H50" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="I50" s="6" t="inlineStr">
+        <is>
+          <t>1M</t>
+        </is>
+      </c>
+      <c r="J50" s="6" t="inlineStr">
+        <is>
+          <t>Approx date; current top frontier model</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2038,7 +4163,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2412,13 +4537,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2790,6 +4915,116 @@
       <c r="D19" s="5" t="inlineStr">
         <is>
           <t>https://github.com/BerriAI/litellm</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>API pricing (GPT-5.x family)</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>https://openai.com/api/pricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Claude API pricing</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>https://www.anthropic.com/pricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Gemini Developer API pricing</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>https://ai.google.dev/gemini-api/docs/pricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>xAI</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Grok API pricing</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>https://docs.x.ai/docs/models</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Models &amp; pricing</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>https://api-docs.deepseek.com/quick_start/pricing</t>
         </is>
       </c>
     </row>
@@ -2810,6 +5045,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>